<commit_message>
100%: thesis backup, finishing section 6.3
</commit_message>
<xml_diff>
--- a/predictions/naive.xlsx
+++ b/predictions/naive.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\denis\Documents\Studies\RTU\Bakalaurs\praktiska-dala\predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D5916BB-A769-4B93-8528-4C8A4F37DE54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C308BCD5-0DA3-44E0-854B-F27E2B9E2734}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1188,6 +1188,14 @@
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F23">
+        <f>AVERAGE(F2:F22)</f>
+        <v>1.7169523809523808</v>
+      </c>
+      <c r="G23">
+        <f>SQRT(AVERAGE(G2:G22))</f>
+        <v>3.7307601676563751</v>
+      </c>
       <c r="H23" s="1">
         <f>AVERAGEA(H2:H22)</f>
         <v>1.2293846153846155</v>

</xml_diff>